<commit_message>
docs: separate frontend and backend Excel artifacts and add Job Summary tables to GitHub Actions
</commit_message>
<xml_diff>
--- a/backend_test_report.xlsx
+++ b/backend_test_report.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="K2" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="K3" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="K4" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="K8" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="K10" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="K12" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="K14" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="K16" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="K18" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="K20" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="K21" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K22" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="K23" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="K24" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="K25" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="K26" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="K27" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="K28" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="K29" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="K30" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="K31" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="K32" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="K33" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="K34" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="K35" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="K36" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="K37" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="K38" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="K39" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:40</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="K40" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="K41" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="K42" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K43" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="K44" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="K45" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="K46" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="K47" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="K48" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="K49" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="K50" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="K51" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="K52" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="K53" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="K54" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="K55" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="K56" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="K57" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="K58" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="K59" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="K60" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="K61" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="K62" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="K63" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="K64" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="K65" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="K66" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="K67" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="K68" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="K69" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="K70" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="K71" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K72" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:40</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="K73" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="K74" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="K75" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="K76" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="K77" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="K78" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="K79" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="K80" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="K81" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="K82" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5800,7 +5800,7 @@
       </c>
       <c r="K83" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="K84" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="K85" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -5974,7 +5974,7 @@
       </c>
       <c r="K86" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="K87" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="K88" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="K89" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="K90" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="K91" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="K92" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="K93" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6439,7 @@
       </c>
       <c r="K94" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="K95" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="K96" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="K97" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="K98" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="K99" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="K100" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>
@@ -6846,7 +6846,7 @@
       </c>
       <c r="K101" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:04:41</t>
+          <t>2026-06-18 14:18:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: bundle markdown report summaries alongside Excel sheets inside frontend and backend artifacts
</commit_message>
<xml_diff>
--- a/backend_test_report.xlsx
+++ b/backend_test_report.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:43</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="K2" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="K3" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="K4" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="K8" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="K10" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="K12" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="K14" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="K16" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="K18" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="K20" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="K21" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K22" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="K23" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="K24" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="K25" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="K26" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="K27" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="K28" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="K29" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="K30" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="K31" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="K32" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="K33" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="K34" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="K35" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="K36" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="K37" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="K38" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="K39" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:40</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="K40" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="K41" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="K42" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K43" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="K44" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="K45" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="K46" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="K47" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="K48" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="K49" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="K50" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="K51" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="K52" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="K53" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="K54" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="K55" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="K56" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="K57" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="K58" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="K59" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="K60" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="K61" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="K62" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="K63" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="K64" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="K65" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="K66" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="K67" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="K68" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="K69" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="K70" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="K71" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K72" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="K73" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="K74" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:41</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="K75" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="K76" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="K77" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="K78" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="K79" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="K80" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="K81" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="K82" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5800,7 +5800,7 @@
       </c>
       <c r="K83" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="K84" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="K85" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -5974,7 +5974,7 @@
       </c>
       <c r="K86" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="K87" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="K88" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="K89" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="K90" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="K91" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="K92" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="K93" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6439,7 @@
       </c>
       <c r="K94" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="K95" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="K96" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="K97" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="K98" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="K99" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="K100" s="18" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>
@@ -6846,7 +6846,7 @@
       </c>
       <c r="K101" s="21" t="inlineStr">
         <is>
-          <t>2026-06-18 14:18:41</t>
+          <t>2026-06-18 19:57:42</t>
         </is>
       </c>
     </row>

</xml_diff>